<commit_message>
data: hourly update 2026-07-10 19:47Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-10.xlsx
+++ b/data/output/workbook/2026-07-10.xlsx
@@ -954,7 +954,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-10 14:32</t>
+          <t>2026-07-10 15:46</t>
         </is>
       </c>
     </row>
@@ -8856,10 +8856,10 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.6506000000000001</v>
+        <v>0.6395999999999999</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-186</v>
+        <v>-177</v>
       </c>
       <c r="H5" s="15" t="n">
         <v>170</v>
@@ -8886,7 +8886,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 65.1% (fair -186). Your call.</t>
+          <t>Model 64.0% (fair -177). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -8898,17 +8898,17 @@
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Cleveland Guardians @ Miami Marlins</t>
+          <t>Houston Astros @ Texas Rangers</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
@@ -8918,17 +8918,17 @@
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Cleveland Guardians +1.5</t>
+          <t>Houston Astros +1.5</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.6058</v>
+        <v>0.6335999999999999</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-154</v>
+        <v>-173</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>186</v>
+        <v>172</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -8952,7 +8952,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 60.6% (fair -154). Your call.</t>
+          <t>Model 63.4% (fair -173). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -8964,17 +8964,17 @@
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Houston Astros @ Texas Rangers</t>
+          <t>Cleveland Guardians @ Miami Marlins</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -8984,17 +8984,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Houston Astros +1.5</t>
+          <t>Cleveland Guardians +1.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.6335999999999999</v>
+        <v>0.6166</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-173</v>
+        <v>-161</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -9018,7 +9018,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 63.4% (fair -173). Your call.</t>
+          <t>Model 61.7% (fair -161). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -9054,13 +9054,13 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.6117</v>
+        <v>0.5977</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-158</v>
+        <v>-149</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -9084,7 +9084,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 61.2% (fair -158). Your call.</t>
+          <t>Model 59.8% (fair -149). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -9101,32 +9101,32 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Boston Red Sox @ New York Mets</t>
+          <t>Milwaukee Brewers @ Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>23:15</t>
+          <t>22:40</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Milwaukee Brewers +1.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.5601</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-217</v>
+        <v>-127</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>125</v>
+        <v>168</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -9150,7 +9150,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 68.5% (fair -217). Your call.</t>
+          <t>Model 56.0% (fair -127). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -9167,32 +9167,32 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers @ Pittsburgh Pirates</t>
+          <t>Boston Red Sox @ New York Mets</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>22:40</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers +1.5</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5694</v>
+        <v>0.6556999999999999</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-132</v>
+        <v>-190</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>170</v>
+        <v>127</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -9216,7 +9216,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 56.9% (fair -132). Your call.</t>
+          <t>Model 65.6% (fair -190). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -9252,10 +9252,10 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.6225000000000001</v>
+        <v>0.6214999999999999</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-165</v>
+        <v>-164</v>
       </c>
       <c r="H11" s="15" t="n">
         <v>138</v>
@@ -9282,7 +9282,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 62.3% (fair -165). Your call.</t>
+          <t>Model 62.1% (fair -164). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -9294,17 +9294,17 @@
     <row r="12">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>Kansas City Royals @ Baltimore Orioles</t>
+          <t>Boston Red Sox @ New York Mets</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="D12" s="20" t="inlineStr">
@@ -9314,17 +9314,17 @@
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>Under 10.5</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.5892999999999999</v>
+        <v>0.6415999999999999</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-143</v>
+        <v>-179</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -9348,7 +9348,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 58.9% (fair -143). Your call.</t>
+          <t>Model 64.2% (fair -179). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -9360,37 +9360,37 @@
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers @ Pittsburgh Pirates</t>
+          <t>Portland Fire @ Atlanta Dream</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>22:40</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Portland Fire</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5762</v>
+        <v>0.1840000000000001</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-136</v>
+        <v>443</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>115</v>
+        <v>614</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -9414,7 +9414,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 57.6% (fair -136). Your call.</t>
+          <t>Model 18.4% (fair +443). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -9426,17 +9426,17 @@
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>Cleveland Guardians @ Miami Marlins</t>
+          <t>Milwaukee Brewers @ Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
@@ -9446,17 +9446,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.5714</v>
+        <v>0.6298</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-133</v>
+        <v>-170</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -9480,7 +9480,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 57.1% (fair -133). Your call.</t>
+          <t>Model 63.0% (fair -170). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -9497,12 +9497,12 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>New York Yankees @ Washington Nationals</t>
+          <t>Kansas City Royals @ Baltimore Orioles</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -9516,13 +9516,13 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.5923</v>
+        <v>0.5801000000000001</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-145</v>
+        <v>-138</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>105</v>
+        <v>123</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 59.2% (fair -145). Your call.</t>
+          <t>Model 58.0% (fair -138). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -9558,37 +9558,37 @@
     <row r="16">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>Portland Fire @ Atlanta Dream</t>
+          <t>Athletics @ Chicago White Sox</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Portland Fire</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.1925</v>
+        <v>0.5564</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>419</v>
+        <v>-125</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>525</v>
+        <v>127</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -9612,7 +9612,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 19.2% (fair +419). Your call.</t>
+          <t>Model 55.6% (fair -125). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -9629,7 +9629,7 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Seattle Mariners @ Tampa Bay Rays</t>
+          <t>Cleveland Guardians @ Miami Marlins</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
@@ -9644,17 +9644,17 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Under 8.5</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.5364</v>
+        <v>0.5712</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-116</v>
+        <v>-133</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -9678,7 +9678,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 53.6% (fair -116). Your call.</t>
+          <t>Model 57.1% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -9705,22 +9705,22 @@
       </c>
       <c r="D18" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates -1.5</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.4306</v>
+        <v>0.5717</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>132</v>
+        <v>-133</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>178</v>
+        <v>115</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -9744,7 +9744,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 43.1% (fair +132). Your call.</t>
+          <t>Model 57.2% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -9761,12 +9761,12 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Athletics @ Chicago White Sox</t>
+          <t>New York Yankees @ Washington Nationals</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -9776,17 +9776,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 9.5</t>
+          <t>Under 10.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.533</v>
+        <v>0.5948</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-114</v>
+        <v>-147</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -9810,7 +9810,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 53.3% (fair -114). Your call.</t>
+          <t>Model 59.5% (fair -147). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -9822,17 +9822,17 @@
     <row r="20">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>Chicago Sky @ Los Angeles Sparks</t>
+          <t>Kansas City Royals @ Baltimore Orioles</t>
         </is>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
@@ -9842,17 +9842,17 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Over 177.5</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.5686</v>
+        <v>0.5749</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>-132</v>
+        <v>-135</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -9876,7 +9876,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 56.9% (fair -132). Your call.</t>
+          <t>Model 57.5% (fair -135). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -9888,37 +9888,37 @@
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>New York Yankees @ Washington Nationals</t>
+          <t>Milwaukee Brewers @ Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>22:40</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Pittsburgh Pirates -1.5</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.5377000000000001</v>
+        <v>0.4399</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>-116</v>
+        <v>127</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>115</v>
+        <v>170</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -9942,7 +9942,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 53.8% (fair -116). Your call.</t>
+          <t>Model 44.0% (fair +127). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -9959,32 +9959,32 @@
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>Dallas Wings @ Toronto Tempo</t>
+          <t>Seattle Mariners @ Tampa Bay Rays</t>
         </is>
       </c>
       <c r="C22" s="20" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D22" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Toronto Tempo</t>
+          <t>Under 8.5</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.288</v>
+        <v>0.5179</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>247</v>
+        <v>-107</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>300</v>
+        <v>125</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -10008,7 +10008,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 28.8% (fair +247). Your call.</t>
+          <t>Model 51.8% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -10020,37 +10020,37 @@
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Kansas City Royals @ Baltimore Orioles</t>
+          <t>Dallas Wings @ Toronto Tempo</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Toronto Tempo</t>
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.5469999999999999</v>
+        <v>0.288</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>-121</v>
+        <v>247</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>110</v>
+        <v>300</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -10074,7 +10074,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 54.7% (fair -121). Your call.</t>
+          <t>Model 28.8% (fair +247). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -10091,32 +10091,32 @@
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>Phoenix Mercury @ Las Vegas Aces</t>
+          <t>Athletics @ Chicago White Sox</t>
         </is>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>Phoenix Mercury</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.2169</v>
+        <v>0.5305</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>361</v>
+        <v>-113</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>426</v>
+        <v>117</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -10140,7 +10140,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 21.7% (fair +361). Your call.</t>
+          <t>Model 53.0% (fair -113). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -10157,32 +10157,32 @@
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>New York Yankees @ Washington Nationals</t>
+          <t>Chicago Sky @ Los Angeles Sparks</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Over 177.5</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.4667</v>
+        <v>0.5735</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>114</v>
+        <v>-134</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>142</v>
+        <v>100</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -10206,7 +10206,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 46.7% (fair +114). Your call.</t>
+          <t>Model 57.4% (fair -134). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -10218,17 +10218,17 @@
     <row r="26">
       <c r="A26" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
-          <t>Cleveland Guardians @ Miami Marlins</t>
+          <t>New York Yankees @ Washington Nationals</t>
         </is>
       </c>
       <c r="C26" s="20" t="inlineStr">
         <is>
-          <t>20:10</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="D26" s="20" t="inlineStr">
@@ -10238,17 +10238,17 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.62</v>
+        <v>0.4658</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>-163</v>
+        <v>115</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>-122</v>
+        <v>144</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -10272,7 +10272,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 62.0% (fair -163). Your call.</t>
+          <t>Model 46.6% (fair +115). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -10284,17 +10284,17 @@
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Dallas Wings @ Toronto Tempo</t>
+          <t>New York Yankees @ Washington Nationals</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
@@ -10304,17 +10304,17 @@
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Over 179.5</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.5291</v>
+        <v>0.5062</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>-112</v>
+        <v>-103</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -10338,7 +10338,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 52.9% (fair -112). Your call.</t>
+          <t>Model 50.6% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -10350,37 +10350,37 @@
     <row r="28">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Houston Astros @ Texas Rangers</t>
+          <t>New York Liberty @ Minnesota Lynx</t>
         </is>
       </c>
       <c r="C28" s="20" t="inlineStr">
         <is>
-          <t>00:05</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Minnesota Lynx -1.5</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.5368000000000001</v>
+        <v>0.5719</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-116</v>
+        <v>-134</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>108</v>
+        <v>-104</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -10404,7 +10404,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 53.7% (fair -116). Your call.</t>
+          <t>Model 57.2% (fair -134). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -10416,12 +10416,12 @@
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Cleveland Guardians @ Miami Marlins</t>
+          <t>Chicago Cubs @ Cincinnati Reds</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
@@ -10431,22 +10431,22 @@
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>Miami Marlins -1.5</t>
+          <t>Over 10.5</t>
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.3942</v>
+        <v>0.5162</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>154</v>
+        <v>-107</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>180</v>
+        <v>117</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -10470,7 +10470,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 39.4% (fair +154). Your call.</t>
+          <t>Model 51.6% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -10647,13 +10647,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4645</v>
+        <v>0.4589</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -10677,7 +10677,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 46.5% (fair +115). Your call.</t>
+          <t>Model 45.9% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -10713,10 +10713,10 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5355</v>
+        <v>0.5411</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-115</v>
+        <v>-118</v>
       </c>
       <c r="H6" s="15" t="n">
         <v>-108</v>
@@ -10743,7 +10743,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 53.5% (fair -115). Your call.</t>
+          <t>Model 54.1% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -10775,17 +10775,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 9</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5236</v>
+        <v>0.5092</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-110</v>
+        <v>-104</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-106</v>
+        <v>105</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -10809,7 +10809,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 52.4% (fair -110). Your call.</t>
+          <t>Model 50.9% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -10841,17 +10841,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 9</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.39</v>
+        <v>0.4908</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>156</v>
+        <v>104</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -10875,7 +10875,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 39.0% (fair +156). Your call.</t>
+          <t>Model 49.1% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -10911,10 +10911,10 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.3883</v>
+        <v>0.4023</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="H9" s="15" t="n">
         <v>178</v>
@@ -10941,7 +10941,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 38.8% (fair +158). Your call.</t>
+          <t>Model 40.2% (fair +149). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -10977,13 +10977,13 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.6117</v>
+        <v>0.5977</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-158</v>
+        <v>-149</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -11007,7 +11007,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 61.2% (fair -158). Your call.</t>
+          <t>Model 59.8% (fair -149). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -11043,13 +11043,13 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.4348</v>
+        <v>0.4251</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -11073,7 +11073,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 43.5% (fair +130). Your call.</t>
+          <t>Model 42.5% (fair +135). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -11109,10 +11109,10 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.5652</v>
+        <v>0.5749</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-130</v>
+        <v>-135</v>
       </c>
       <c r="H12" s="15" t="n">
         <v>-117</v>
@@ -11139,7 +11139,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 56.5% (fair -130). Your call.</t>
+          <t>Model 57.5% (fair -135). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -11175,10 +11175,10 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5762</v>
+        <v>0.5717</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-136</v>
+        <v>-133</v>
       </c>
       <c r="H13" s="15" t="n">
         <v>115</v>
@@ -11205,7 +11205,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 57.6% (fair -136). Your call.</t>
+          <t>Model 57.2% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -11241,10 +11241,10 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4238</v>
+        <v>0.4283</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="H14" s="15" t="n">
         <v>105</v>
@@ -11271,7 +11271,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 42.4% (fair +136). Your call.</t>
+          <t>Model 42.8% (fair +133). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -11307,13 +11307,13 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.4306</v>
+        <v>0.4399</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -11337,7 +11337,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 43.1% (fair +132). Your call.</t>
+          <t>Model 44.0% (fair +127). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -11373,13 +11373,13 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.5694</v>
+        <v>0.5601</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-132</v>
+        <v>-127</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -11403,7 +11403,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 56.9% (fair -132). Your call.</t>
+          <t>Model 56.0% (fair -127). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -11439,10 +11439,10 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.5333</v>
+        <v>0.5342</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-114</v>
+        <v>-115</v>
       </c>
       <c r="H17" s="15" t="n">
         <v>-144</v>
@@ -11469,7 +11469,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 53.3% (fair -114). Your call.</t>
+          <t>Model 53.4% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -11505,13 +11505,13 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.4667</v>
+        <v>0.4658</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -11535,7 +11535,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 46.7% (fair +114). Your call.</t>
+          <t>Model 46.6% (fair +115). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -11571,13 +11571,13 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.4077</v>
+        <v>0.4052</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -11601,7 +11601,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 40.8% (fair +145). Your call.</t>
+          <t>Model 40.5% (fair +147). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -11637,13 +11637,13 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.5923</v>
+        <v>0.5948</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>-145</v>
+        <v>-147</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -11667,7 +11667,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 59.2% (fair -145). Your call.</t>
+          <t>Model 59.5% (fair -147). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -11703,13 +11703,13 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.5649</v>
+        <v>0.5617</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>-130</v>
+        <v>-128</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>-113</v>
+        <v>-108</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -11733,7 +11733,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 56.5% (fair -130). Your call.</t>
+          <t>Model 56.2% (fair -128). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -11769,10 +11769,10 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.4351</v>
+        <v>0.4383</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H22" s="15" t="n">
         <v>108</v>
@@ -11799,7 +11799,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 43.5% (fair +130). Your call.</t>
+          <t>Model 43.8% (fair +128). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -11835,13 +11835,13 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.4227</v>
+        <v>0.4149</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -11865,7 +11865,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 42.3% (fair +137). Your call.</t>
+          <t>Model 41.5% (fair +141). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -11901,13 +11901,13 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5773</v>
+        <v>0.5851</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-137</v>
+        <v>-141</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>-138</v>
+        <v>-134</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -11931,7 +11931,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -137). Your call.</t>
+          <t>Model 58.5% (fair -141). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -11967,10 +11967,10 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.4107</v>
+        <v>0.4199</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="H25" s="15" t="n">
         <v>108</v>
@@ -11997,7 +11997,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 41.1% (fair +143). Your call.</t>
+          <t>Model 42.0% (fair +138). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -12033,13 +12033,13 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.5892999999999999</v>
+        <v>0.5801000000000001</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>-143</v>
+        <v>-138</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -12063,7 +12063,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 58.9% (fair -143). Your call.</t>
+          <t>Model 58.0% (fair -138). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -12099,10 +12099,10 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.4162</v>
+        <v>0.4243</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="H27" s="15" t="n">
         <v>138</v>
@@ -12129,7 +12129,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 41.6% (fair +140). Your call.</t>
+          <t>Model 42.4% (fair +136). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -12165,13 +12165,13 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.5838</v>
+        <v>0.5757</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-140</v>
+        <v>-136</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>-144</v>
+        <v>-141</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -12195,7 +12195,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 58.4% (fair -140). Your call.</t>
+          <t>Model 57.6% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -12231,13 +12231,13 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.5262</v>
+        <v>0.5278</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-111</v>
+        <v>-112</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>-104</v>
+        <v>-106</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -12261,7 +12261,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 52.6% (fair -111). Your call.</t>
+          <t>Model 52.8% (fair -112). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -12297,10 +12297,10 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.4738</v>
+        <v>0.4722</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H30" s="15" t="n">
         <v>104</v>
@@ -12327,7 +12327,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 47.4% (fair +111). Your call.</t>
+          <t>Model 47.2% (fair +112). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>
@@ -12363,10 +12363,10 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.5187</v>
+        <v>0.5205</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>-108</v>
+        <v>-109</v>
       </c>
       <c r="H31" s="15" t="n">
         <v>108</v>
@@ -12393,7 +12393,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 51.9% (fair -108). Your call.</t>
+          <t>Model 52.0% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -12429,13 +12429,13 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.4813</v>
+        <v>0.4795</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>-110</v>
+        <v>-108</v>
       </c>
       <c r="I32" s="13">
         <f>IF($H$32="","",IF($H$32&lt;0,-$H$32/(-$H$32+100),100/($H$32+100)))</f>
@@ -12459,7 +12459,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 48.1% (fair +108). Your call.</t>
+          <t>Model 48.0% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -12495,7 +12495,7 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.5727</v>
+        <v>0.5726</v>
       </c>
       <c r="G33" s="14" t="n">
         <v>-134</v>
@@ -12561,7 +12561,7 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.4273</v>
+        <v>0.4274</v>
       </c>
       <c r="G34" s="14" t="n">
         <v>134</v>
@@ -12627,10 +12627,10 @@
         </is>
       </c>
       <c r="F35" s="13" t="n">
-        <v>0.4696</v>
+        <v>0.4683</v>
       </c>
       <c r="G35" s="14" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H35" s="15" t="n">
         <v>108</v>
@@ -12657,7 +12657,7 @@
       </c>
       <c r="N35" s="19" t="inlineStr">
         <is>
-          <t>Model 47.0% (fair +113). Your call.</t>
+          <t>Model 46.8% (fair +114). Your call.</t>
         </is>
       </c>
       <c r="O35" s="15" t="n"/>
@@ -12693,13 +12693,13 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.5304</v>
+        <v>0.5317</v>
       </c>
       <c r="G36" s="14" t="n">
-        <v>-113</v>
+        <v>-114</v>
       </c>
       <c r="H36" s="15" t="n">
-        <v>-110</v>
+        <v>-111</v>
       </c>
       <c r="I36" s="13">
         <f>IF($H$36="","",IF($H$36&lt;0,-$H$36/(-$H$36+100),100/($H$36+100)))</f>
@@ -12723,7 +12723,7 @@
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>Model 53.0% (fair -113). Your call.</t>
+          <t>Model 53.2% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O36" s="15" t="n"/>
@@ -12759,10 +12759,10 @@
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>0.4636</v>
+        <v>0.4821</v>
       </c>
       <c r="G37" s="14" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="H37" s="15" t="n">
         <v>113</v>
@@ -12789,7 +12789,7 @@
       </c>
       <c r="N37" s="19" t="inlineStr">
         <is>
-          <t>Model 46.4% (fair +116). Your call.</t>
+          <t>Model 48.2% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O37" s="15" t="n"/>
@@ -12825,13 +12825,13 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.5364</v>
+        <v>0.5179</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>-116</v>
+        <v>-107</v>
       </c>
       <c r="H38" s="15" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I38" s="13">
         <f>IF($H$38="","",IF($H$38&lt;0,-$H$38/(-$H$38+100),100/($H$38+100)))</f>
@@ -12855,7 +12855,7 @@
       </c>
       <c r="N38" s="19" t="inlineStr">
         <is>
-          <t>Model 53.6% (fair -116). Your call.</t>
+          <t>Model 51.8% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O38" s="15" t="n"/>
@@ -12891,13 +12891,13 @@
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>0.3494</v>
+        <v>0.3604</v>
       </c>
       <c r="G39" s="14" t="n">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="H39" s="15" t="n">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="I39" s="13">
         <f>IF($H$39="","",IF($H$39&lt;0,-$H$39/(-$H$39+100),100/($H$39+100)))</f>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>Model 34.9% (fair +186). Your call.</t>
+          <t>Model 36.0% (fair +177). Your call.</t>
         </is>
       </c>
       <c r="O39" s="15" t="n"/>
@@ -12957,10 +12957,10 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.6506000000000001</v>
+        <v>0.6395999999999999</v>
       </c>
       <c r="G40" s="14" t="n">
-        <v>-186</v>
+        <v>-177</v>
       </c>
       <c r="H40" s="15" t="n">
         <v>170</v>
@@ -12987,7 +12987,7 @@
       </c>
       <c r="N40" s="19" t="inlineStr">
         <is>
-          <t>Model 65.1% (fair -186). Your call.</t>
+          <t>Model 64.0% (fair -177). Your call.</t>
         </is>
       </c>
       <c r="O40" s="15" t="n"/>
@@ -13023,13 +13023,13 @@
         </is>
       </c>
       <c r="F41" s="13" t="n">
-        <v>0.4528</v>
+        <v>0.4524</v>
       </c>
       <c r="G41" s="14" t="n">
         <v>121</v>
       </c>
       <c r="H41" s="15" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I41" s="13">
         <f>IF($H$41="","",IF($H$41&lt;0,-$H$41/(-$H$41+100),100/($H$41+100)))</f>
@@ -13053,7 +13053,7 @@
       </c>
       <c r="N41" s="19" t="inlineStr">
         <is>
-          <t>Model 45.3% (fair +121). Your call.</t>
+          <t>Model 45.2% (fair +121). Your call.</t>
         </is>
       </c>
       <c r="O41" s="15" t="n"/>
@@ -13089,7 +13089,7 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.5472</v>
+        <v>0.5476</v>
       </c>
       <c r="G42" s="14" t="n">
         <v>-121</v>
@@ -13119,7 +13119,7 @@
       </c>
       <c r="N42" s="19" t="inlineStr">
         <is>
-          <t>Model 54.7% (fair -121). Your call.</t>
+          <t>Model 54.8% (fair -121). Your call.</t>
         </is>
       </c>
       <c r="O42" s="15" t="n"/>
@@ -13155,13 +13155,13 @@
         </is>
       </c>
       <c r="F43" s="13" t="n">
-        <v>0.5714</v>
+        <v>0.5712</v>
       </c>
       <c r="G43" s="14" t="n">
         <v>-133</v>
       </c>
       <c r="H43" s="15" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="I43" s="13">
         <f>IF($H$43="","",IF($H$43&lt;0,-$H$43/(-$H$43+100),100/($H$43+100)))</f>
@@ -13221,13 +13221,13 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.4286</v>
+        <v>0.4288</v>
       </c>
       <c r="G44" s="14" t="n">
         <v>133</v>
       </c>
       <c r="H44" s="15" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="I44" s="13">
         <f>IF($H$44="","",IF($H$44&lt;0,-$H$44/(-$H$44+100),100/($H$44+100)))</f>
@@ -13287,10 +13287,10 @@
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>0.3942</v>
+        <v>0.3834</v>
       </c>
       <c r="G45" s="14" t="n">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="H45" s="15" t="n">
         <v>180</v>
@@ -13317,7 +13317,7 @@
       </c>
       <c r="N45" s="19" t="inlineStr">
         <is>
-          <t>Model 39.4% (fair +154). Your call.</t>
+          <t>Model 38.3% (fair +161). Your call.</t>
         </is>
       </c>
       <c r="O45" s="15" t="n"/>
@@ -13353,13 +13353,13 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.6058</v>
+        <v>0.6166</v>
       </c>
       <c r="G46" s="14" t="n">
-        <v>-154</v>
+        <v>-161</v>
       </c>
       <c r="H46" s="15" t="n">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="I46" s="13">
         <f>IF($H$46="","",IF($H$46&lt;0,-$H$46/(-$H$46+100),100/($H$46+100)))</f>
@@ -13383,7 +13383,7 @@
       </c>
       <c r="N46" s="19" t="inlineStr">
         <is>
-          <t>Model 60.6% (fair -154). Your call.</t>
+          <t>Model 61.7% (fair -161). Your call.</t>
         </is>
       </c>
       <c r="O46" s="15" t="n"/>
@@ -13419,13 +13419,13 @@
         </is>
       </c>
       <c r="F47" s="13" t="n">
-        <v>0.4222</v>
+        <v>0.4252</v>
       </c>
       <c r="G47" s="14" t="n">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="H47" s="15" t="n">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I47" s="13">
         <f>IF($H$47="","",IF($H$47&lt;0,-$H$47/(-$H$47+100),100/($H$47+100)))</f>
@@ -13449,7 +13449,7 @@
       </c>
       <c r="N47" s="19" t="inlineStr">
         <is>
-          <t>Model 42.2% (fair +137). Your call.</t>
+          <t>Model 42.5% (fair +135). Your call.</t>
         </is>
       </c>
       <c r="O47" s="15" t="n"/>
@@ -13485,10 +13485,10 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.5778</v>
+        <v>0.5748</v>
       </c>
       <c r="G48" s="14" t="n">
-        <v>-137</v>
+        <v>-135</v>
       </c>
       <c r="H48" s="15" t="n">
         <v>-138</v>
@@ -13515,7 +13515,7 @@
       </c>
       <c r="N48" s="19" t="inlineStr">
         <is>
-          <t>Model 57.8% (fair -137). Your call.</t>
+          <t>Model 57.5% (fair -135). Your call.</t>
         </is>
       </c>
       <c r="O48" s="15" t="n"/>
@@ -13551,13 +13551,13 @@
         </is>
       </c>
       <c r="F49" s="13" t="n">
-        <v>0.315</v>
+        <v>0.3443</v>
       </c>
       <c r="G49" s="14" t="n">
-        <v>217</v>
+        <v>190</v>
       </c>
       <c r="H49" s="15" t="n">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="I49" s="13">
         <f>IF($H$49="","",IF($H$49&lt;0,-$H$49/(-$H$49+100),100/($H$49+100)))</f>
@@ -13581,7 +13581,7 @@
       </c>
       <c r="N49" s="19" t="inlineStr">
         <is>
-          <t>Model 31.5% (fair +217). Your call.</t>
+          <t>Model 34.4% (fair +190). Your call.</t>
         </is>
       </c>
       <c r="O49" s="15" t="n"/>
@@ -13617,13 +13617,13 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.6556999999999999</v>
       </c>
       <c r="G50" s="14" t="n">
-        <v>-217</v>
+        <v>-190</v>
       </c>
       <c r="H50" s="15" t="n">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I50" s="13">
         <f>IF($H$50="","",IF($H$50&lt;0,-$H$50/(-$H$50+100),100/($H$50+100)))</f>
@@ -13647,7 +13647,7 @@
       </c>
       <c r="N50" s="19" t="inlineStr">
         <is>
-          <t>Model 68.5% (fair -217). Your call.</t>
+          <t>Model 65.6% (fair -190). Your call.</t>
         </is>
       </c>
       <c r="O50" s="15" t="n"/>
@@ -13683,13 +13683,13 @@
         </is>
       </c>
       <c r="F51" s="13" t="n">
-        <v>0.3775</v>
+        <v>0.3785</v>
       </c>
       <c r="G51" s="14" t="n">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H51" s="15" t="n">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="I51" s="13">
         <f>IF($H$51="","",IF($H$51&lt;0,-$H$51/(-$H$51+100),100/($H$51+100)))</f>
@@ -13713,7 +13713,7 @@
       </c>
       <c r="N51" s="19" t="inlineStr">
         <is>
-          <t>Model 37.8% (fair +165). Your call.</t>
+          <t>Model 37.9% (fair +164). Your call.</t>
         </is>
       </c>
       <c r="O51" s="15" t="n"/>
@@ -13749,10 +13749,10 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.6225000000000001</v>
+        <v>0.6214999999999999</v>
       </c>
       <c r="G52" s="14" t="n">
-        <v>-165</v>
+        <v>-164</v>
       </c>
       <c r="H52" s="15" t="n">
         <v>138</v>
@@ -13779,7 +13779,7 @@
       </c>
       <c r="N52" s="19" t="inlineStr">
         <is>
-          <t>Model 62.3% (fair -165). Your call.</t>
+          <t>Model 62.1% (fair -164). Your call.</t>
         </is>
       </c>
       <c r="O52" s="15" t="n"/>
@@ -13815,10 +13815,10 @@
         </is>
       </c>
       <c r="F53" s="13" t="n">
-        <v>0.3587399999999999</v>
+        <v>0.25926</v>
       </c>
       <c r="G53" s="14" t="n">
-        <v>179</v>
+        <v>286</v>
       </c>
       <c r="H53" s="15" t="n">
         <v>144</v>
@@ -13845,7 +13845,7 @@
       </c>
       <c r="N53" s="19" t="inlineStr">
         <is>
-          <t>Model 35.9% (fair +179). Your call.</t>
+          <t>Model 25.9% (fair +286). Your call.</t>
         </is>
       </c>
       <c r="O53" s="15" t="n"/>
@@ -13881,13 +13881,13 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.6412600000000001</v>
+        <v>0.74074</v>
       </c>
       <c r="G54" s="14" t="n">
-        <v>-179</v>
+        <v>-286</v>
       </c>
       <c r="H54" s="15" t="n">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I54" s="13">
         <f>IF($H$54="","",IF($H$54&lt;0,-$H$54/(-$H$54+100),100/($H$54+100)))</f>
@@ -13911,7 +13911,7 @@
       </c>
       <c r="N54" s="19" t="inlineStr">
         <is>
-          <t>Model 64.1% (fair -179). Your call.</t>
+          <t>Model 74.1% (fair -286). Your call.</t>
         </is>
       </c>
       <c r="O54" s="15" t="n"/>
@@ -13947,13 +13947,13 @@
         </is>
       </c>
       <c r="F55" s="13" t="n">
-        <v>0.533</v>
+        <v>0.5564</v>
       </c>
       <c r="G55" s="14" t="n">
-        <v>-114</v>
+        <v>-125</v>
       </c>
       <c r="H55" s="15" t="n">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="I55" s="13">
         <f>IF($H$55="","",IF($H$55&lt;0,-$H$55/(-$H$55+100),100/($H$55+100)))</f>
@@ -13977,7 +13977,7 @@
       </c>
       <c r="N55" s="19" t="inlineStr">
         <is>
-          <t>Model 53.3% (fair -114). Your call.</t>
+          <t>Model 55.6% (fair -125). Your call.</t>
         </is>
       </c>
       <c r="O55" s="15" t="n"/>
@@ -14013,13 +14013,13 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.467</v>
+        <v>0.4436</v>
       </c>
       <c r="G56" s="14" t="n">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="H56" s="15" t="n">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I56" s="13">
         <f>IF($H$56="","",IF($H$56&lt;0,-$H$56/(-$H$56+100),100/($H$56+100)))</f>
@@ -14043,7 +14043,7 @@
       </c>
       <c r="N56" s="19" t="inlineStr">
         <is>
-          <t>Model 46.7% (fair +114). Your call.</t>
+          <t>Model 44.4% (fair +125). Your call.</t>
         </is>
       </c>
       <c r="O56" s="15" t="n"/>
@@ -14079,10 +14079,10 @@
         </is>
       </c>
       <c r="F57" s="13" t="n">
-        <v>0.4312</v>
+        <v>0.4394</v>
       </c>
       <c r="G57" s="14" t="n">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="H57" s="15" t="n">
         <v>138</v>
@@ -14109,7 +14109,7 @@
       </c>
       <c r="N57" s="19" t="inlineStr">
         <is>
-          <t>Model 43.1% (fair +132). Your call.</t>
+          <t>Model 43.9% (fair +128). Your call.</t>
         </is>
       </c>
       <c r="O57" s="15" t="n"/>
@@ -14145,10 +14145,10 @@
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.5688</v>
+        <v>0.5606</v>
       </c>
       <c r="G58" s="14" t="n">
-        <v>-132</v>
+        <v>-128</v>
       </c>
       <c r="H58" s="15" t="n">
         <v>-141</v>
@@ -14175,7 +14175,7 @@
       </c>
       <c r="N58" s="19" t="inlineStr">
         <is>
-          <t>Model 56.9% (fair -132). Your call.</t>
+          <t>Model 56.1% (fair -128). Your call.</t>
         </is>
       </c>
       <c r="O58" s="15" t="n"/>
@@ -14211,13 +14211,13 @@
         </is>
       </c>
       <c r="F59" s="13" t="n">
-        <v>0.5206999999999999</v>
+        <v>0.5212</v>
       </c>
       <c r="G59" s="14" t="n">
         <v>-109</v>
       </c>
       <c r="H59" s="15" t="n">
-        <v>-132</v>
+        <v>-133</v>
       </c>
       <c r="I59" s="13">
         <f>IF($H$59="","",IF($H$59&lt;0,-$H$59/(-$H$59+100),100/($H$59+100)))</f>
@@ -14277,7 +14277,7 @@
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.4793</v>
+        <v>0.4788</v>
       </c>
       <c r="G60" s="14" t="n">
         <v>109</v>
@@ -14343,13 +14343,13 @@
         </is>
       </c>
       <c r="F61" s="13" t="n">
-        <v>0.5368000000000001</v>
+        <v>0.5065</v>
       </c>
       <c r="G61" s="14" t="n">
-        <v>-116</v>
+        <v>-103</v>
       </c>
       <c r="H61" s="15" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I61" s="13">
         <f>IF($H$61="","",IF($H$61&lt;0,-$H$61/(-$H$61+100),100/($H$61+100)))</f>
@@ -14373,7 +14373,7 @@
       </c>
       <c r="N61" s="19" t="inlineStr">
         <is>
-          <t>Model 53.7% (fair -116). Your call.</t>
+          <t>Model 50.6% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O61" s="15" t="n"/>
@@ -14409,13 +14409,13 @@
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>0.4631999999999999</v>
+        <v>0.4935</v>
       </c>
       <c r="G62" s="14" t="n">
-        <v>116</v>
+        <v>103</v>
       </c>
       <c r="H62" s="15" t="n">
-        <v>110</v>
+        <v>-104</v>
       </c>
       <c r="I62" s="13">
         <f>IF($H$62="","",IF($H$62&lt;0,-$H$62/(-$H$62+100),100/($H$62+100)))</f>
@@ -14439,7 +14439,7 @@
       </c>
       <c r="N62" s="19" t="inlineStr">
         <is>
-          <t>Model 46.3% (fair +116). Your call.</t>
+          <t>Model 49.4% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O62" s="15" t="n"/>
@@ -14607,10 +14607,10 @@
         </is>
       </c>
       <c r="F65" s="13" t="n">
-        <v>0.4293</v>
+        <v>0.4251</v>
       </c>
       <c r="G65" s="14" t="n">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H65" s="15" t="n"/>
       <c r="I65" s="13">
@@ -14635,7 +14635,7 @@
       </c>
       <c r="N65" s="19" t="inlineStr">
         <is>
-          <t>Model 42.9% (fair +133). Your call.</t>
+          <t>Model 42.5% (fair +135). Your call.</t>
         </is>
       </c>
       <c r="O65" s="15" t="n"/>
@@ -14671,10 +14671,10 @@
         </is>
       </c>
       <c r="F66" s="13" t="n">
-        <v>0.5707</v>
+        <v>0.5749</v>
       </c>
       <c r="G66" s="14" t="n">
-        <v>-133</v>
+        <v>-135</v>
       </c>
       <c r="H66" s="15" t="n"/>
       <c r="I66" s="13">
@@ -14699,7 +14699,7 @@
       </c>
       <c r="N66" s="19" t="inlineStr">
         <is>
-          <t>Model 57.1% (fair -133). Your call.</t>
+          <t>Model 57.5% (fair -135). Your call.</t>
         </is>
       </c>
       <c r="O66" s="15" t="n"/>
@@ -14735,10 +14735,10 @@
         </is>
       </c>
       <c r="F67" s="13" t="n">
-        <v>0.5197000000000001</v>
+        <v>0.5152</v>
       </c>
       <c r="G67" s="14" t="n">
-        <v>-108</v>
+        <v>-106</v>
       </c>
       <c r="H67" s="15" t="n"/>
       <c r="I67" s="13">
@@ -14763,7 +14763,7 @@
       </c>
       <c r="N67" s="19" t="inlineStr">
         <is>
-          <t>Model 52.0% (fair -108). Your call.</t>
+          <t>Model 51.5% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O67" s="15" t="n"/>
@@ -14799,10 +14799,10 @@
         </is>
       </c>
       <c r="F68" s="13" t="n">
-        <v>0.4803</v>
+        <v>0.4848</v>
       </c>
       <c r="G68" s="14" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H68" s="15" t="n"/>
       <c r="I68" s="13">
@@ -14827,7 +14827,7 @@
       </c>
       <c r="N68" s="19" t="inlineStr">
         <is>
-          <t>Model 48.0% (fair +108). Your call.</t>
+          <t>Model 48.5% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O68" s="15" t="n"/>
@@ -14863,7 +14863,7 @@
         </is>
       </c>
       <c r="F69" s="13" t="n">
-        <v>0.4201</v>
+        <v>0.4195</v>
       </c>
       <c r="G69" s="14" t="n">
         <v>138</v>
@@ -14891,7 +14891,7 @@
       </c>
       <c r="N69" s="19" t="inlineStr">
         <is>
-          <t>Model 42.0% (fair +138). Your call.</t>
+          <t>Model 41.9% (fair +138). Your call.</t>
         </is>
       </c>
       <c r="O69" s="15" t="n"/>
@@ -14927,7 +14927,7 @@
         </is>
       </c>
       <c r="F70" s="13" t="n">
-        <v>0.5799</v>
+        <v>0.5805</v>
       </c>
       <c r="G70" s="14" t="n">
         <v>-138</v>
@@ -14955,7 +14955,7 @@
       </c>
       <c r="N70" s="19" t="inlineStr">
         <is>
-          <t>Model 58.0% (fair -138). Your call.</t>
+          <t>Model 58.1% (fair -138). Your call.</t>
         </is>
       </c>
       <c r="O70" s="15" t="n"/>
@@ -14991,10 +14991,10 @@
         </is>
       </c>
       <c r="F71" s="13" t="n">
-        <v>0.365</v>
+        <v>0.3631</v>
       </c>
       <c r="G71" s="14" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H71" s="15" t="n"/>
       <c r="I71" s="13">
@@ -15019,7 +15019,7 @@
       </c>
       <c r="N71" s="19" t="inlineStr">
         <is>
-          <t>Model 36.5% (fair +174). Your call.</t>
+          <t>Model 36.3% (fair +175). Your call.</t>
         </is>
       </c>
       <c r="O71" s="15" t="n"/>
@@ -15055,10 +15055,10 @@
         </is>
       </c>
       <c r="F72" s="13" t="n">
-        <v>0.635</v>
+        <v>0.6369</v>
       </c>
       <c r="G72" s="14" t="n">
-        <v>-174</v>
+        <v>-175</v>
       </c>
       <c r="H72" s="15" t="n"/>
       <c r="I72" s="13">
@@ -15083,7 +15083,7 @@
       </c>
       <c r="N72" s="19" t="inlineStr">
         <is>
-          <t>Model 63.5% (fair -174). Your call.</t>
+          <t>Model 63.7% (fair -175). Your call.</t>
         </is>
       </c>
       <c r="O72" s="15" t="n"/>
@@ -15119,7 +15119,7 @@
         </is>
       </c>
       <c r="F73" s="13" t="n">
-        <v>0.5069</v>
+        <v>0.5063</v>
       </c>
       <c r="G73" s="14" t="n">
         <v>-103</v>
@@ -15147,7 +15147,7 @@
       </c>
       <c r="N73" s="19" t="inlineStr">
         <is>
-          <t>Model 50.7% (fair -103). Your call.</t>
+          <t>Model 50.6% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O73" s="15" t="n"/>
@@ -15183,7 +15183,7 @@
         </is>
       </c>
       <c r="F74" s="13" t="n">
-        <v>0.4932</v>
+        <v>0.4937</v>
       </c>
       <c r="G74" s="14" t="n">
         <v>103</v>
@@ -15211,7 +15211,7 @@
       </c>
       <c r="N74" s="19" t="inlineStr">
         <is>
-          <t>Model 49.3% (fair +103). Your call.</t>
+          <t>Model 49.4% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O74" s="15" t="n"/>
@@ -15247,10 +15247,10 @@
         </is>
       </c>
       <c r="F75" s="13" t="n">
-        <v>0.3504</v>
+        <v>0.3379</v>
       </c>
       <c r="G75" s="14" t="n">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="H75" s="15" t="n">
         <v>163</v>
@@ -15277,7 +15277,7 @@
       </c>
       <c r="N75" s="19" t="inlineStr">
         <is>
-          <t>Model 35.0% (fair +185). Your call.</t>
+          <t>Model 33.8% (fair +196). Your call.</t>
         </is>
       </c>
       <c r="O75" s="15" t="n"/>
@@ -15313,10 +15313,10 @@
         </is>
       </c>
       <c r="F76" s="13" t="n">
-        <v>0.6496</v>
+        <v>0.6621</v>
       </c>
       <c r="G76" s="14" t="n">
-        <v>-185</v>
+        <v>-196</v>
       </c>
       <c r="H76" s="15" t="n">
         <v>-163</v>
@@ -15343,7 +15343,7 @@
       </c>
       <c r="N76" s="19" t="inlineStr">
         <is>
-          <t>Model 65.0% (fair -185). Your call.</t>
+          <t>Model 66.2% (fair -196). Your call.</t>
         </is>
       </c>
       <c r="O76" s="15" t="n"/>
@@ -15451,7 +15451,7 @@
         <v>114</v>
       </c>
       <c r="H78" s="15" t="n">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="I78" s="13">
         <f>IF($H$78="","",IF($H$78&lt;0,-$H$78/(-$H$78+100),100/($H$78+100)))</f>
@@ -15507,17 +15507,17 @@
       </c>
       <c r="E79" s="12" t="inlineStr">
         <is>
-          <t>Over 9</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F79" s="13" t="n">
-        <v>0.4952</v>
+        <v>0.5305</v>
       </c>
       <c r="G79" s="14" t="n">
-        <v>102</v>
+        <v>-113</v>
       </c>
       <c r="H79" s="15" t="n">
-        <v>-110</v>
+        <v>117</v>
       </c>
       <c r="I79" s="13">
         <f>IF($H$79="","",IF($H$79&lt;0,-$H$79/(-$H$79+100),100/($H$79+100)))</f>
@@ -15541,7 +15541,7 @@
       </c>
       <c r="N79" s="19" t="inlineStr">
         <is>
-          <t>Model 49.5% (fair +102). Your call.</t>
+          <t>Model 53.0% (fair -113). Your call.</t>
         </is>
       </c>
       <c r="O79" s="15" t="n"/>
@@ -15573,14 +15573,14 @@
       </c>
       <c r="E80" s="20" t="inlineStr">
         <is>
-          <t>Under 9</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F80" s="13" t="n">
-        <v>0.4182</v>
+        <v>0.4695</v>
       </c>
       <c r="G80" s="14" t="n">
-        <v>139</v>
+        <v>113</v>
       </c>
       <c r="H80" s="15" t="n">
         <v>115</v>
@@ -15607,7 +15607,7 @@
       </c>
       <c r="N80" s="19" t="inlineStr">
         <is>
-          <t>Model 41.8% (fair +139). Your call.</t>
+          <t>Model 47.0% (fair +113). Your call.</t>
         </is>
       </c>
       <c r="O80" s="15" t="n"/>
@@ -15643,13 +15643,13 @@
         </is>
       </c>
       <c r="F81" s="13" t="n">
-        <v>0.5873</v>
+        <v>0.5859</v>
       </c>
       <c r="G81" s="14" t="n">
-        <v>-142</v>
+        <v>-141</v>
       </c>
       <c r="H81" s="15" t="n">
-        <v>-170</v>
+        <v>-165</v>
       </c>
       <c r="I81" s="13">
         <f>IF($H$81="","",IF($H$81&lt;0,-$H$81/(-$H$81+100),100/($H$81+100)))</f>
@@ -15673,7 +15673,7 @@
       </c>
       <c r="N81" s="19" t="inlineStr">
         <is>
-          <t>Model 58.7% (fair -142). Your call.</t>
+          <t>Model 58.6% (fair -141). Your call.</t>
         </is>
       </c>
       <c r="O81" s="15" t="n"/>
@@ -15709,10 +15709,10 @@
         </is>
       </c>
       <c r="F82" s="13" t="n">
-        <v>0.4127</v>
+        <v>0.4141</v>
       </c>
       <c r="G82" s="14" t="n">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H82" s="15" t="n">
         <v>145</v>
@@ -15739,7 +15739,7 @@
       </c>
       <c r="N82" s="19" t="inlineStr">
         <is>
-          <t>Model 41.3% (fair +142). Your call.</t>
+          <t>Model 41.4% (fair +141). Your call.</t>
         </is>
       </c>
       <c r="O82" s="15" t="n"/>
@@ -15775,13 +15775,13 @@
         </is>
       </c>
       <c r="F83" s="13" t="n">
-        <v>0.4345</v>
+        <v>0.4338</v>
       </c>
       <c r="G83" s="14" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H83" s="15" t="n">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="I83" s="13">
         <f>IF($H$83="","",IF($H$83&lt;0,-$H$83/(-$H$83+100),100/($H$83+100)))</f>
@@ -15805,7 +15805,7 @@
       </c>
       <c r="N83" s="19" t="inlineStr">
         <is>
-          <t>Model 43.5% (fair +130). Your call.</t>
+          <t>Model 43.4% (fair +131). Your call.</t>
         </is>
       </c>
       <c r="O83" s="15" t="n"/>
@@ -15841,13 +15841,13 @@
         </is>
       </c>
       <c r="F84" s="13" t="n">
-        <v>0.5655</v>
+        <v>0.5662</v>
       </c>
       <c r="G84" s="14" t="n">
-        <v>-130</v>
+        <v>-131</v>
       </c>
       <c r="H84" s="15" t="n">
-        <v>-130</v>
+        <v>-138</v>
       </c>
       <c r="I84" s="13">
         <f>IF($H$84="","",IF($H$84&lt;0,-$H$84/(-$H$84+100),100/($H$84+100)))</f>
@@ -15871,7 +15871,7 @@
       </c>
       <c r="N84" s="19" t="inlineStr">
         <is>
-          <t>Model 56.5% (fair -130). Your call.</t>
+          <t>Model 56.6% (fair -131). Your call.</t>
         </is>
       </c>
       <c r="O84" s="15" t="n"/>
@@ -15907,10 +15907,10 @@
         </is>
       </c>
       <c r="F85" s="13" t="n">
-        <v>0.5085</v>
+        <v>0.5099</v>
       </c>
       <c r="G85" s="14" t="n">
-        <v>-103</v>
+        <v>-104</v>
       </c>
       <c r="H85" s="15" t="n">
         <v>105</v>
@@ -15937,7 +15937,7 @@
       </c>
       <c r="N85" s="19" t="inlineStr">
         <is>
-          <t>Model 50.8% (fair -103). Your call.</t>
+          <t>Model 51.0% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O85" s="15" t="n"/>
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F86" s="13" t="n">
-        <v>0.4915</v>
+        <v>0.4901</v>
       </c>
       <c r="G86" s="14" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H86" s="15" t="n">
-        <v>-110</v>
+        <v>-108</v>
       </c>
       <c r="I86" s="13">
         <f>IF($H$86="","",IF($H$86&lt;0,-$H$86/(-$H$86+100),100/($H$86+100)))</f>
@@ -16003,7 +16003,7 @@
       </c>
       <c r="N86" s="19" t="inlineStr">
         <is>
-          <t>Model 49.2% (fair +103). Your call.</t>
+          <t>Model 49.0% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O86" s="15" t="n"/>
@@ -16039,10 +16039,10 @@
         </is>
       </c>
       <c r="F87" s="13" t="n">
-        <v>0.3765</v>
+        <v>0.3801</v>
       </c>
       <c r="G87" s="14" t="n">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="H87" s="15" t="n">
         <v>160</v>
@@ -16069,7 +16069,7 @@
       </c>
       <c r="N87" s="19" t="inlineStr">
         <is>
-          <t>Model 37.6% (fair +166). Your call.</t>
+          <t>Model 38.0% (fair +163). Your call.</t>
         </is>
       </c>
       <c r="O87" s="15" t="n"/>
@@ -16105,13 +16105,13 @@
         </is>
       </c>
       <c r="F88" s="13" t="n">
-        <v>0.6234999999999999</v>
+        <v>0.6199</v>
       </c>
       <c r="G88" s="14" t="n">
-        <v>-166</v>
+        <v>-163</v>
       </c>
       <c r="H88" s="15" t="n">
-        <v>-170</v>
+        <v>-160</v>
       </c>
       <c r="I88" s="13">
         <f>IF($H$88="","",IF($H$88&lt;0,-$H$88/(-$H$88+100),100/($H$88+100)))</f>
@@ -16135,7 +16135,7 @@
       </c>
       <c r="N88" s="19" t="inlineStr">
         <is>
-          <t>Model 62.3% (fair -166). Your call.</t>
+          <t>Model 62.0% (fair -163). Your call.</t>
         </is>
       </c>
       <c r="O88" s="15" t="n"/>
@@ -16171,13 +16171,13 @@
         </is>
       </c>
       <c r="F89" s="13" t="n">
-        <v>0.5933999999999999</v>
+        <v>0.5977</v>
       </c>
       <c r="G89" s="14" t="n">
-        <v>-146</v>
+        <v>-149</v>
       </c>
       <c r="H89" s="15" t="n">
-        <v>-156</v>
+        <v>-163</v>
       </c>
       <c r="I89" s="13">
         <f>IF($H$89="","",IF($H$89&lt;0,-$H$89/(-$H$89+100),100/($H$89+100)))</f>
@@ -16201,7 +16201,7 @@
       </c>
       <c r="N89" s="19" t="inlineStr">
         <is>
-          <t>Model 59.3% (fair -146). Your call.</t>
+          <t>Model 59.8% (fair -149). Your call.</t>
         </is>
       </c>
       <c r="O89" s="15" t="n"/>
@@ -16237,13 +16237,13 @@
         </is>
       </c>
       <c r="F90" s="13" t="n">
-        <v>0.4066</v>
+        <v>0.4023</v>
       </c>
       <c r="G90" s="14" t="n">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="H90" s="15" t="n">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="I90" s="13">
         <f>IF($H$90="","",IF($H$90&lt;0,-$H$90/(-$H$90+100),100/($H$90+100)))</f>
@@ -16267,7 +16267,7 @@
       </c>
       <c r="N90" s="19" t="inlineStr">
         <is>
-          <t>Model 40.7% (fair +146). Your call.</t>
+          <t>Model 40.2% (fair +149). Your call.</t>
         </is>
       </c>
       <c r="O90" s="15" t="n"/>
@@ -16303,13 +16303,13 @@
         </is>
       </c>
       <c r="F91" s="13" t="n">
-        <v>0.4623</v>
+        <v>0.5062</v>
       </c>
       <c r="G91" s="14" t="n">
-        <v>116</v>
+        <v>-103</v>
       </c>
       <c r="H91" s="15" t="n">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="I91" s="13">
         <f>IF($H$91="","",IF($H$91&lt;0,-$H$91/(-$H$91+100),100/($H$91+100)))</f>
@@ -16333,7 +16333,7 @@
       </c>
       <c r="N91" s="19" t="inlineStr">
         <is>
-          <t>Model 46.2% (fair +116). Your call.</t>
+          <t>Model 50.6% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O91" s="15" t="n"/>
@@ -16369,10 +16369,10 @@
         </is>
       </c>
       <c r="F92" s="13" t="n">
-        <v>0.5377000000000001</v>
+        <v>0.4938</v>
       </c>
       <c r="G92" s="14" t="n">
-        <v>-116</v>
+        <v>103</v>
       </c>
       <c r="H92" s="15" t="n">
         <v>115</v>
@@ -16399,7 +16399,7 @@
       </c>
       <c r="N92" s="19" t="inlineStr">
         <is>
-          <t>Model 53.8% (fair -116). Your call.</t>
+          <t>Model 49.4% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O92" s="15" t="n"/>
@@ -16435,7 +16435,7 @@
         </is>
       </c>
       <c r="F93" s="13" t="n">
-        <v>0.4955</v>
+        <v>0.4956</v>
       </c>
       <c r="G93" s="14" t="n">
         <v>102</v>
@@ -16465,7 +16465,7 @@
       </c>
       <c r="N93" s="19" t="inlineStr">
         <is>
-          <t>Model 49.5% (fair +102). Your call.</t>
+          <t>Model 49.6% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O93" s="15" t="n"/>
@@ -16501,13 +16501,13 @@
         </is>
       </c>
       <c r="F94" s="13" t="n">
-        <v>0.5044999999999999</v>
+        <v>0.5044</v>
       </c>
       <c r="G94" s="14" t="n">
         <v>-102</v>
       </c>
       <c r="H94" s="15" t="n">
-        <v>-114</v>
+        <v>-110</v>
       </c>
       <c r="I94" s="13">
         <f>IF($H$94="","",IF($H$94&lt;0,-$H$94/(-$H$94+100),100/($H$94+100)))</f>
@@ -16567,7 +16567,7 @@
         </is>
       </c>
       <c r="F95" s="13" t="n">
-        <v>0.5041</v>
+        <v>0.5056</v>
       </c>
       <c r="G95" s="14" t="n">
         <v>-102</v>
@@ -16597,7 +16597,7 @@
       </c>
       <c r="N95" s="19" t="inlineStr">
         <is>
-          <t>Model 50.4% (fair -102). Your call.</t>
+          <t>Model 50.6% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O95" s="15" t="n"/>
@@ -16633,13 +16633,13 @@
         </is>
       </c>
       <c r="F96" s="13" t="n">
-        <v>0.4959</v>
+        <v>0.4944</v>
       </c>
       <c r="G96" s="14" t="n">
         <v>102</v>
       </c>
       <c r="H96" s="15" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="I96" s="13">
         <f>IF($H$96="","",IF($H$96&lt;0,-$H$96/(-$H$96+100),100/($H$96+100)))</f>
@@ -16663,7 +16663,7 @@
       </c>
       <c r="N96" s="19" t="inlineStr">
         <is>
-          <t>Model 49.6% (fair +102). Your call.</t>
+          <t>Model 49.4% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O96" s="15" t="n"/>
@@ -16699,13 +16699,13 @@
         </is>
       </c>
       <c r="F97" s="13" t="n">
-        <v>0.5636</v>
+        <v>0.6298</v>
       </c>
       <c r="G97" s="14" t="n">
-        <v>-129</v>
+        <v>-170</v>
       </c>
       <c r="H97" s="15" t="n">
-        <v>-120</v>
+        <v>108</v>
       </c>
       <c r="I97" s="13">
         <f>IF($H$97="","",IF($H$97&lt;0,-$H$97/(-$H$97+100),100/($H$97+100)))</f>
@@ -16729,7 +16729,7 @@
       </c>
       <c r="N97" s="19" t="inlineStr">
         <is>
-          <t>Model 56.4% (fair -129). Your call.</t>
+          <t>Model 63.0% (fair -170). Your call.</t>
         </is>
       </c>
       <c r="O97" s="15" t="n"/>
@@ -16765,10 +16765,10 @@
         </is>
       </c>
       <c r="F98" s="13" t="n">
-        <v>0.4364</v>
+        <v>0.3702</v>
       </c>
       <c r="G98" s="14" t="n">
-        <v>129</v>
+        <v>170</v>
       </c>
       <c r="H98" s="15" t="n">
         <v>105</v>
@@ -16795,7 +16795,7 @@
       </c>
       <c r="N98" s="19" t="inlineStr">
         <is>
-          <t>Model 43.6% (fair +129). Your call.</t>
+          <t>Model 37.0% (fair +170). Your call.</t>
         </is>
       </c>
       <c r="O98" s="15" t="n"/>
@@ -16963,13 +16963,13 @@
         </is>
       </c>
       <c r="F101" s="13" t="n">
-        <v>0.4370000000000001</v>
+        <v>0.4302</v>
       </c>
       <c r="G101" s="14" t="n">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="H101" s="15" t="n">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="I101" s="13">
         <f>IF($H$101="","",IF($H$101&lt;0,-$H$101/(-$H$101+100),100/($H$101+100)))</f>
@@ -16993,7 +16993,7 @@
       </c>
       <c r="N101" s="19" t="inlineStr">
         <is>
-          <t>Model 43.7% (fair +129). Your call.</t>
+          <t>Model 43.0% (fair +132). Your call.</t>
         </is>
       </c>
       <c r="O101" s="15" t="n"/>
@@ -17029,13 +17029,13 @@
         </is>
       </c>
       <c r="F102" s="13" t="n">
-        <v>0.5629999999999999</v>
+        <v>0.5698</v>
       </c>
       <c r="G102" s="14" t="n">
-        <v>-129</v>
+        <v>-132</v>
       </c>
       <c r="H102" s="15" t="n">
-        <v>-127</v>
+        <v>-133</v>
       </c>
       <c r="I102" s="13">
         <f>IF($H$102="","",IF($H$102&lt;0,-$H$102/(-$H$102+100),100/($H$102+100)))</f>
@@ -17059,7 +17059,7 @@
       </c>
       <c r="N102" s="19" t="inlineStr">
         <is>
-          <t>Model 56.3% (fair -129). Your call.</t>
+          <t>Model 57.0% (fair -132). Your call.</t>
         </is>
       </c>
       <c r="O102" s="15" t="n"/>
@@ -17091,17 +17091,17 @@
       </c>
       <c r="E103" s="12" t="inlineStr">
         <is>
-          <t>Over 9</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F103" s="13" t="n">
-        <v>0.441</v>
+        <v>0.3584</v>
       </c>
       <c r="G103" s="14" t="n">
-        <v>127</v>
+        <v>179</v>
       </c>
       <c r="H103" s="15" t="n">
-        <v>-110</v>
+        <v>117</v>
       </c>
       <c r="I103" s="13">
         <f>IF($H$103="","",IF($H$103&lt;0,-$H$103/(-$H$103+100),100/($H$103+100)))</f>
@@ -17125,7 +17125,7 @@
       </c>
       <c r="N103" s="19" t="inlineStr">
         <is>
-          <t>Model 44.1% (fair +127). Your call.</t>
+          <t>Model 35.8% (fair +179). Your call.</t>
         </is>
       </c>
       <c r="O103" s="15" t="n"/>
@@ -17157,14 +17157,14 @@
       </c>
       <c r="E104" s="20" t="inlineStr">
         <is>
-          <t>Under 9</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F104" s="13" t="n">
-        <v>0.4757</v>
+        <v>0.6415999999999999</v>
       </c>
       <c r="G104" s="14" t="n">
-        <v>110</v>
+        <v>-179</v>
       </c>
       <c r="H104" s="15" t="n">
         <v>115</v>
@@ -17191,7 +17191,7 @@
       </c>
       <c r="N104" s="19" t="inlineStr">
         <is>
-          <t>Model 47.6% (fair +110). Your call.</t>
+          <t>Model 64.2% (fair -179). Your call.</t>
         </is>
       </c>
       <c r="O104" s="15" t="n"/>
@@ -17227,10 +17227,10 @@
         </is>
       </c>
       <c r="F105" s="13" t="n">
-        <v>0.4765</v>
+        <v>0.4786</v>
       </c>
       <c r="G105" s="14" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H105" s="15" t="n">
         <v>113</v>
@@ -17257,7 +17257,7 @@
       </c>
       <c r="N105" s="19" t="inlineStr">
         <is>
-          <t>Model 47.7% (fair +110). Your call.</t>
+          <t>Model 47.9% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O105" s="15" t="n"/>
@@ -17293,13 +17293,13 @@
         </is>
       </c>
       <c r="F106" s="13" t="n">
-        <v>0.5235</v>
+        <v>0.5214</v>
       </c>
       <c r="G106" s="14" t="n">
+        <v>-109</v>
+      </c>
+      <c r="H106" s="15" t="n">
         <v>-110</v>
-      </c>
-      <c r="H106" s="15" t="n">
-        <v>-113</v>
       </c>
       <c r="I106" s="13">
         <f>IF($H$106="","",IF($H$106&lt;0,-$H$106/(-$H$106+100),100/($H$106+100)))</f>
@@ -17323,7 +17323,7 @@
       </c>
       <c r="N106" s="19" t="inlineStr">
         <is>
-          <t>Model 52.3% (fair -110). Your call.</t>
+          <t>Model 52.1% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O106" s="15" t="n"/>
@@ -17359,13 +17359,13 @@
         </is>
       </c>
       <c r="F107" s="13" t="n">
-        <v>0.5014999999999999</v>
+        <v>0.5094</v>
       </c>
       <c r="G107" s="14" t="n">
-        <v>-101</v>
+        <v>-104</v>
       </c>
       <c r="H107" s="15" t="n">
-        <v>100</v>
+        <v>-104</v>
       </c>
       <c r="I107" s="13">
         <f>IF($H$107="","",IF($H$107&lt;0,-$H$107/(-$H$107+100),100/($H$107+100)))</f>
@@ -17389,7 +17389,7 @@
       </c>
       <c r="N107" s="19" t="inlineStr">
         <is>
-          <t>Model 50.1% (fair -101). Your call.</t>
+          <t>Model 50.9% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O107" s="15" t="n"/>
@@ -17425,13 +17425,13 @@
         </is>
       </c>
       <c r="F108" s="13" t="n">
-        <v>0.4985000000000001</v>
+        <v>0.4906</v>
       </c>
       <c r="G108" s="14" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="H108" s="15" t="n">
-        <v>-115</v>
+        <v>-108</v>
       </c>
       <c r="I108" s="13">
         <f>IF($H$108="","",IF($H$108&lt;0,-$H$108/(-$H$108+100),100/($H$108+100)))</f>
@@ -17455,7 +17455,7 @@
       </c>
       <c r="N108" s="19" t="inlineStr">
         <is>
-          <t>Model 49.9% (fair +101). Your call.</t>
+          <t>Model 49.1% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O108" s="15" t="n"/>
@@ -17491,13 +17491,13 @@
         </is>
       </c>
       <c r="F109" s="13" t="n">
-        <v>0.6222</v>
+        <v>0.6209</v>
       </c>
       <c r="G109" s="14" t="n">
-        <v>-165</v>
+        <v>-164</v>
       </c>
       <c r="H109" s="15" t="n">
-        <v>-195</v>
+        <v>-190</v>
       </c>
       <c r="I109" s="13">
         <f>IF($H$109="","",IF($H$109&lt;0,-$H$109/(-$H$109+100),100/($H$109+100)))</f>
@@ -17521,7 +17521,7 @@
       </c>
       <c r="N109" s="19" t="inlineStr">
         <is>
-          <t>Model 62.2% (fair -165). Your call.</t>
+          <t>Model 62.1% (fair -164). Your call.</t>
         </is>
       </c>
       <c r="O109" s="15" t="n"/>
@@ -17557,10 +17557,10 @@
         </is>
       </c>
       <c r="F110" s="13" t="n">
-        <v>0.3778</v>
+        <v>0.3791</v>
       </c>
       <c r="G110" s="14" t="n">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H110" s="15" t="n">
         <v>165</v>
@@ -17587,7 +17587,7 @@
       </c>
       <c r="N110" s="19" t="inlineStr">
         <is>
-          <t>Model 37.8% (fair +165). Your call.</t>
+          <t>Model 37.9% (fair +164). Your call.</t>
         </is>
       </c>
       <c r="O110" s="15" t="n"/>
@@ -17623,10 +17623,10 @@
         </is>
       </c>
       <c r="F111" s="13" t="n">
-        <v>0.38</v>
+        <v>0.3771</v>
       </c>
       <c r="G111" s="14" t="n">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="H111" s="15" t="n">
         <v>127</v>
@@ -17653,7 +17653,7 @@
       </c>
       <c r="N111" s="19" t="inlineStr">
         <is>
-          <t>Model 38.0% (fair +163). Your call.</t>
+          <t>Model 37.7% (fair +165). Your call.</t>
         </is>
       </c>
       <c r="O111" s="15" t="n"/>
@@ -17689,13 +17689,13 @@
         </is>
       </c>
       <c r="F112" s="13" t="n">
-        <v>0.62</v>
+        <v>0.6229</v>
       </c>
       <c r="G112" s="14" t="n">
-        <v>-163</v>
+        <v>-165</v>
       </c>
       <c r="H112" s="15" t="n">
-        <v>-122</v>
+        <v>-127</v>
       </c>
       <c r="I112" s="13">
         <f>IF($H$112="","",IF($H$112&lt;0,-$H$112/(-$H$112+100),100/($H$112+100)))</f>
@@ -17719,7 +17719,7 @@
       </c>
       <c r="N112" s="19" t="inlineStr">
         <is>
-          <t>Model 62.0% (fair -163). Your call.</t>
+          <t>Model 62.3% (fair -165). Your call.</t>
         </is>
       </c>
       <c r="O112" s="15" t="n"/>
@@ -17755,10 +17755,10 @@
         </is>
       </c>
       <c r="F113" s="13" t="n">
-        <v>0.4958</v>
+        <v>0.5016</v>
       </c>
       <c r="G113" s="14" t="n">
-        <v>102</v>
+        <v>-101</v>
       </c>
       <c r="H113" s="15" t="n">
         <v>-105</v>
@@ -17785,7 +17785,7 @@
       </c>
       <c r="N113" s="19" t="inlineStr">
         <is>
-          <t>Model 49.6% (fair +102). Your call.</t>
+          <t>Model 50.2% (fair -101). Your call.</t>
         </is>
       </c>
       <c r="O113" s="15" t="n"/>
@@ -17821,13 +17821,13 @@
         </is>
       </c>
       <c r="F114" s="13" t="n">
-        <v>0.4139</v>
+        <v>0.4081</v>
       </c>
       <c r="G114" s="14" t="n">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="H114" s="15" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="I114" s="13">
         <f>IF($H$114="","",IF($H$114&lt;0,-$H$114/(-$H$114+100),100/($H$114+100)))</f>
@@ -17851,7 +17851,7 @@
       </c>
       <c r="N114" s="19" t="inlineStr">
         <is>
-          <t>Model 41.4% (fair +142). Your call.</t>
+          <t>Model 40.8% (fair +145). Your call.</t>
         </is>
       </c>
       <c r="O114" s="15" t="n"/>
@@ -17887,10 +17887,10 @@
         </is>
       </c>
       <c r="F115" s="13" t="n">
-        <v>0.4124</v>
+        <v>0.4142</v>
       </c>
       <c r="G115" s="14" t="n">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H115" s="15" t="n">
         <v>160</v>
@@ -17917,7 +17917,7 @@
       </c>
       <c r="N115" s="19" t="inlineStr">
         <is>
-          <t>Model 41.2% (fair +142). Your call.</t>
+          <t>Model 41.4% (fair +141). Your call.</t>
         </is>
       </c>
       <c r="O115" s="15" t="n"/>
@@ -17953,13 +17953,13 @@
         </is>
       </c>
       <c r="F116" s="13" t="n">
-        <v>0.5876</v>
+        <v>0.5858</v>
       </c>
       <c r="G116" s="14" t="n">
-        <v>-142</v>
+        <v>-141</v>
       </c>
       <c r="H116" s="15" t="n">
-        <v>-170</v>
+        <v>-165</v>
       </c>
       <c r="I116" s="13">
         <f>IF($H$116="","",IF($H$116&lt;0,-$H$116/(-$H$116+100),100/($H$116+100)))</f>
@@ -17983,7 +17983,7 @@
       </c>
       <c r="N116" s="19" t="inlineStr">
         <is>
-          <t>Model 58.8% (fair -142). Your call.</t>
+          <t>Model 58.6% (fair -141). Your call.</t>
         </is>
       </c>
       <c r="O116" s="15" t="n"/>
@@ -18151,13 +18151,13 @@
         </is>
       </c>
       <c r="F119" s="13" t="n">
-        <v>0.5256</v>
+        <v>0.5101</v>
       </c>
       <c r="G119" s="14" t="n">
-        <v>-111</v>
+        <v>-104</v>
       </c>
       <c r="H119" s="15" t="n">
-        <v>-106</v>
+        <v>105</v>
       </c>
       <c r="I119" s="13">
         <f>IF($H$119="","",IF($H$119&lt;0,-$H$119/(-$H$119+100),100/($H$119+100)))</f>
@@ -18181,7 +18181,7 @@
       </c>
       <c r="N119" s="19" t="inlineStr">
         <is>
-          <t>Model 52.6% (fair -111). Your call.</t>
+          <t>Model 51.0% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O119" s="15" t="n"/>
@@ -18217,13 +18217,13 @@
         </is>
       </c>
       <c r="F120" s="13" t="n">
-        <v>0.4744</v>
+        <v>0.4899</v>
       </c>
       <c r="G120" s="14" t="n">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="H120" s="15" t="n">
-        <v>-110</v>
+        <v>100</v>
       </c>
       <c r="I120" s="13">
         <f>IF($H$120="","",IF($H$120&lt;0,-$H$120/(-$H$120+100),100/($H$120+100)))</f>
@@ -18247,7 +18247,7 @@
       </c>
       <c r="N120" s="19" t="inlineStr">
         <is>
-          <t>Model 47.4% (fair +111). Your call.</t>
+          <t>Model 49.0% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O120" s="15" t="n"/>
@@ -18283,10 +18283,10 @@
         </is>
       </c>
       <c r="F121" s="13" t="n">
-        <v>0.5766</v>
+        <v>0.5815</v>
       </c>
       <c r="G121" s="14" t="n">
-        <v>-136</v>
+        <v>-139</v>
       </c>
       <c r="H121" s="15" t="n">
         <v>-130</v>
@@ -18313,7 +18313,7 @@
       </c>
       <c r="N121" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
+          <t>Model 58.1% (fair -139). Your call.</t>
         </is>
       </c>
       <c r="O121" s="15" t="n"/>
@@ -18349,13 +18349,13 @@
         </is>
       </c>
       <c r="F122" s="13" t="n">
-        <v>0.4234</v>
+        <v>0.4185</v>
       </c>
       <c r="G122" s="14" t="n">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="H122" s="15" t="n">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="I122" s="13">
         <f>IF($H$122="","",IF($H$122&lt;0,-$H$122/(-$H$122+100),100/($H$122+100)))</f>
@@ -18379,7 +18379,7 @@
       </c>
       <c r="N122" s="19" t="inlineStr">
         <is>
-          <t>Model 42.3% (fair +136). Your call.</t>
+          <t>Model 41.9% (fair +139). Your call.</t>
         </is>
       </c>
       <c r="O122" s="15" t="n"/>
@@ -18547,10 +18547,10 @@
         </is>
       </c>
       <c r="F125" s="13" t="n">
-        <v>0.453</v>
+        <v>0.4251</v>
       </c>
       <c r="G125" s="14" t="n">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="H125" s="15" t="n">
         <v>104</v>
@@ -18577,7 +18577,7 @@
       </c>
       <c r="N125" s="19" t="inlineStr">
         <is>
-          <t>Model 45.3% (fair +121). Your call.</t>
+          <t>Model 42.5% (fair +135). Your call.</t>
         </is>
       </c>
       <c r="O125" s="15" t="n"/>
@@ -18613,10 +18613,10 @@
         </is>
       </c>
       <c r="F126" s="13" t="n">
-        <v>0.5469999999999999</v>
+        <v>0.5749</v>
       </c>
       <c r="G126" s="14" t="n">
-        <v>-121</v>
+        <v>-135</v>
       </c>
       <c r="H126" s="15" t="n">
         <v>110</v>
@@ -18643,7 +18643,7 @@
       </c>
       <c r="N126" s="19" t="inlineStr">
         <is>
-          <t>Model 54.7% (fair -121). Your call.</t>
+          <t>Model 57.5% (fair -135). Your call.</t>
         </is>
       </c>
       <c r="O126" s="15" t="n"/>
@@ -18679,10 +18679,10 @@
         </is>
       </c>
       <c r="F127" s="13" t="n">
-        <v>0.409</v>
+        <v>0.4066</v>
       </c>
       <c r="G127" s="14" t="n">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="H127" s="15" t="n">
         <v>140</v>
@@ -18709,7 +18709,7 @@
       </c>
       <c r="N127" s="19" t="inlineStr">
         <is>
-          <t>Model 40.9% (fair +144). Your call.</t>
+          <t>Model 40.7% (fair +146). Your call.</t>
         </is>
       </c>
       <c r="O127" s="15" t="n"/>
@@ -18745,10 +18745,10 @@
         </is>
       </c>
       <c r="F128" s="13" t="n">
-        <v>0.591</v>
+        <v>0.5933999999999999</v>
       </c>
       <c r="G128" s="14" t="n">
-        <v>-144</v>
+        <v>-146</v>
       </c>
       <c r="H128" s="15" t="n">
         <v>-145</v>
@@ -18775,7 +18775,7 @@
       </c>
       <c r="N128" s="19" t="inlineStr">
         <is>
-          <t>Model 59.1% (fair -144). Your call.</t>
+          <t>Model 59.3% (fair -146). Your call.</t>
         </is>
       </c>
       <c r="O128" s="15" t="n"/>
@@ -18939,10 +18939,10 @@
         </is>
       </c>
       <c r="F131" s="13" t="n">
-        <v>0.51</v>
+        <v>0.5114</v>
       </c>
       <c r="G131" s="14" t="n">
-        <v>-104</v>
+        <v>-105</v>
       </c>
       <c r="H131" s="15" t="n">
         <v>-105</v>
@@ -18969,7 +18969,7 @@
       </c>
       <c r="N131" s="19" t="inlineStr">
         <is>
-          <t>Model 51.0% (fair -104). Your call.</t>
+          <t>Model 51.1% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O131" s="15" t="n"/>
@@ -19005,13 +19005,13 @@
         </is>
       </c>
       <c r="F132" s="13" t="n">
-        <v>0.49</v>
+        <v>0.4886</v>
       </c>
       <c r="G132" s="14" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H132" s="15" t="n">
-        <v>-110</v>
+        <v>-108</v>
       </c>
       <c r="I132" s="13">
         <f>IF($H$132="","",IF($H$132&lt;0,-$H$132/(-$H$132+100),100/($H$132+100)))</f>
@@ -19035,7 +19035,7 @@
       </c>
       <c r="N132" s="19" t="inlineStr">
         <is>
-          <t>Model 49.0% (fair +104). Your call.</t>
+          <t>Model 48.9% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O132" s="15" t="n"/>
@@ -19331,13 +19331,13 @@
         </is>
       </c>
       <c r="F137" s="13" t="n">
-        <v>0.5132</v>
+        <v>0.5162</v>
       </c>
       <c r="G137" s="14" t="n">
-        <v>-105</v>
+        <v>-107</v>
       </c>
       <c r="H137" s="15" t="n">
-        <v>-110</v>
+        <v>117</v>
       </c>
       <c r="I137" s="13">
         <f>IF($H$137="","",IF($H$137&lt;0,-$H$137/(-$H$137+100),100/($H$137+100)))</f>
@@ -19361,7 +19361,7 @@
       </c>
       <c r="N137" s="19" t="inlineStr">
         <is>
-          <t>Model 51.3% (fair -105). Your call.</t>
+          <t>Model 51.6% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O137" s="15" t="n"/>
@@ -19397,10 +19397,10 @@
         </is>
       </c>
       <c r="F138" s="13" t="n">
-        <v>0.4868</v>
+        <v>0.4838</v>
       </c>
       <c r="G138" s="14" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H138" s="15" t="n">
         <v>100</v>
@@ -19427,7 +19427,7 @@
       </c>
       <c r="N138" s="19" t="inlineStr">
         <is>
-          <t>Model 48.7% (fair +105). Your call.</t>
+          <t>Model 48.4% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O138" s="15" t="n"/>
@@ -19463,7 +19463,7 @@
         </is>
       </c>
       <c r="F139" s="13" t="n">
-        <v>0.5628</v>
+        <v>0.5641</v>
       </c>
       <c r="G139" s="14" t="n">
         <v>-129</v>
@@ -19493,7 +19493,7 @@
       </c>
       <c r="N139" s="19" t="inlineStr">
         <is>
-          <t>Model 56.3% (fair -129). Your call.</t>
+          <t>Model 56.4% (fair -129). Your call.</t>
         </is>
       </c>
       <c r="O139" s="15" t="n"/>
@@ -19529,13 +19529,13 @@
         </is>
       </c>
       <c r="F140" s="13" t="n">
-        <v>0.4372</v>
+        <v>0.4359</v>
       </c>
       <c r="G140" s="14" t="n">
         <v>129</v>
       </c>
       <c r="H140" s="15" t="n">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="I140" s="13">
         <f>IF($H$140="","",IF($H$140&lt;0,-$H$140/(-$H$140+100),100/($H$140+100)))</f>
@@ -19559,7 +19559,7 @@
       </c>
       <c r="N140" s="19" t="inlineStr">
         <is>
-          <t>Model 43.7% (fair +129). Your call.</t>
+          <t>Model 43.6% (fair +129). Your call.</t>
         </is>
       </c>
       <c r="O140" s="15" t="n"/>
@@ -20120,10 +20120,10 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.7178</v>
+        <v>0.7188</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-254</v>
+        <v>-256</v>
       </c>
       <c r="H5" s="15" t="n">
         <v>-233</v>
@@ -20150,7 +20150,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 71.8% (fair -254). Your call.</t>
+          <t>Model 71.9% (fair -256). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -20186,13 +20186,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.2822</v>
+        <v>0.2812</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -20216,7 +20216,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 28.2% (fair +254). Your call.</t>
+          <t>Model 28.1% (fair +256). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -20648,10 +20648,10 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5291</v>
+        <v>0.5833957033370806</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-112</v>
+        <v>-140</v>
       </c>
       <c r="H13" s="15" t="n">
         <v>113</v>
@@ -20678,7 +20678,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 52.9% (fair -112). Your call.</t>
+          <t>Model 58.3% (fair -140). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -20714,13 +20714,13 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4709</v>
+        <v>0.4166042966629194</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>112</v>
+        <v>140</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>-108</v>
+        <v>-103</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -20744,7 +20744,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 47.1% (fair +112). Your call.</t>
+          <t>Model 41.7% (fair +140). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -20786,7 +20786,7 @@
         <v>-153</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -20912,13 +20912,13 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4448</v>
+        <v>0.4391</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -20942,7 +20942,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 44.5% (fair +125). Your call.</t>
+          <t>Model 43.9% (fair +128). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -20978,13 +20978,13 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5552</v>
+        <v>0.5609</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-125</v>
+        <v>-128</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>-108</v>
+        <v>-113</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -21008,7 +21008,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 55.5% (fair -125). Your call.</t>
+          <t>Model 56.1% (fair -128). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -21044,13 +21044,13 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5686</v>
+        <v>0.5735</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-132</v>
+        <v>-134</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -21074,7 +21074,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 56.9% (fair -132). Your call.</t>
+          <t>Model 57.4% (fair -134). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -21110,10 +21110,10 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4314</v>
+        <v>0.4265</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="H20" s="15" t="n">
         <v>100</v>
@@ -21140,7 +21140,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 43.1% (fair +132). Your call.</t>
+          <t>Model 42.6% (fair +134). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -21308,13 +21308,13 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.3287474</v>
+        <v>0.3895999999999999</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>204</v>
+        <v>157</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -21338,7 +21338,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 32.9% (fair +204). Your call.</t>
+          <t>Model 39.0% (fair +157). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -21374,10 +21374,10 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.6712526</v>
+        <v>0.6104000000000001</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-204</v>
+        <v>-157</v>
       </c>
       <c r="H24" s="15" t="n">
         <v>-122</v>
@@ -21404,7 +21404,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 67.1% (fair -204). Your call.</t>
+          <t>Model 61.0% (fair -157). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -21568,17 +21568,17 @@
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Minnesota Lynx -2.5</t>
+          <t>Minnesota Lynx -1.5</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.5558</v>
+        <v>0.5719</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>-125</v>
+        <v>-134</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>-102</v>
+        <v>-104</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -21602,7 +21602,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 55.6% (fair -125). Your call.</t>
+          <t>Model 57.2% (fair -134). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -21634,14 +21634,14 @@
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>New York Liberty +2.5</t>
+          <t>New York Liberty +1.5</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.4442</v>
+        <v>0.4281</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="H28" s="15" t="n">
         <v>100</v>
@@ -21668,7 +21668,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 44.4% (fair +125). Your call.</t>
+          <t>Model 42.8% (fair +134). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -21704,13 +21704,13 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.1925</v>
+        <v>0.1840000000000001</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>419</v>
+        <v>443</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>525</v>
+        <v>614</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -21734,7 +21734,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 19.2% (fair +419). Your call.</t>
+          <t>Model 18.4% (fair +443). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -21770,10 +21770,10 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.8075</v>
+        <v>0.8159999999999999</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-419</v>
+        <v>-443</v>
       </c>
       <c r="H30" s="15" t="n">
         <v>-567</v>
@@ -21800,7 +21800,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 80.8% (fair -419). Your call.</t>
+          <t>Model 81.6% (fair -443). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>
@@ -21968,13 +21968,13 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.3926414967183107</v>
+        <v>0.4337</v>
       </c>
       <c r="G33" s="14" t="n">
-        <v>155</v>
+        <v>131</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="I33" s="13">
         <f>IF($H$33="","",IF($H$33&lt;0,-$H$33/(-$H$33+100),100/($H$33+100)))</f>
@@ -21998,7 +21998,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Model 39.3% (fair +155). Your call.</t>
+          <t>Model 43.4% (fair +131). Your call.</t>
         </is>
       </c>
       <c r="O33" s="15" t="n"/>
@@ -22034,13 +22034,13 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.6073585032816893</v>
+        <v>0.5663</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>-155</v>
+        <v>-131</v>
       </c>
       <c r="H34" s="15" t="n">
-        <v>-105</v>
+        <v>-108</v>
       </c>
       <c r="I34" s="13">
         <f>IF($H$34="","",IF($H$34&lt;0,-$H$34/(-$H$34+100),100/($H$34+100)))</f>
@@ -22064,7 +22064,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Model 60.7% (fair -155). Your call.</t>
+          <t>Model 56.6% (fair -131). Your call.</t>
         </is>
       </c>
       <c r="O34" s="15" t="n"/>
@@ -22100,13 +22100,13 @@
         </is>
       </c>
       <c r="F35" s="13" t="n">
-        <v>0.2169</v>
+        <v>0.2205</v>
       </c>
       <c r="G35" s="14" t="n">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="H35" s="15" t="n">
-        <v>426</v>
+        <v>400</v>
       </c>
       <c r="I35" s="13">
         <f>IF($H$35="","",IF($H$35&lt;0,-$H$35/(-$H$35+100),100/($H$35+100)))</f>
@@ -22130,7 +22130,7 @@
       </c>
       <c r="N35" s="19" t="inlineStr">
         <is>
-          <t>Model 21.7% (fair +361). Your call.</t>
+          <t>Model 22.1% (fair +354). Your call.</t>
         </is>
       </c>
       <c r="O35" s="15" t="n"/>
@@ -22166,13 +22166,13 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.7831</v>
+        <v>0.7795</v>
       </c>
       <c r="G36" s="14" t="n">
-        <v>-361</v>
+        <v>-354</v>
       </c>
       <c r="H36" s="15" t="n">
-        <v>-413</v>
+        <v>-425</v>
       </c>
       <c r="I36" s="13">
         <f>IF($H$36="","",IF($H$36&lt;0,-$H$36/(-$H$36+100),100/($H$36+100)))</f>
@@ -22196,7 +22196,7 @@
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>Model 78.3% (fair -361). Your call.</t>
+          <t>Model 78.0% (fair -354). Your call.</t>
         </is>
       </c>
       <c r="O36" s="15" t="n"/>

</xml_diff>